<commit_message>
New implementation to calculate feed requirements (only cattle done, other livestock will fail)
</commit_message>
<xml_diff>
--- a/mini/data/default/CattleHerd.xlsx
+++ b/mini/data/default/CattleHerd.xlsx
@@ -144,7 +144,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2370" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2401" uniqueCount="603">
   <si>
     <t>value</t>
   </si>
@@ -1922,6 +1922,39 @@
   </si>
   <si>
     <t>Assumed same as for beef</t>
+  </si>
+  <si>
+    <t>Energy</t>
+  </si>
+  <si>
+    <t>Protein (AAT)</t>
+  </si>
+  <si>
+    <t>AAT_factor</t>
+  </si>
+  <si>
+    <t>g AAT/MJ ME</t>
+  </si>
+  <si>
+    <t>Spörndly (2003). Tabell 5</t>
+  </si>
+  <si>
+    <t>Rough for now… 7.5 @ 40-75 kg LW … 6.5 @ &gt;275 kg LW</t>
+  </si>
+  <si>
+    <t>Dry matter intake</t>
+  </si>
+  <si>
+    <t>max_DMI</t>
+  </si>
+  <si>
+    <t>https://pir.sa.gov.au/__data/assets/pdf_file/0007/272869/Calculating_dry_matter_intakes.pdf</t>
+  </si>
+  <si>
+    <t>kg DM/head/day</t>
+  </si>
+  <si>
+    <t>handle pre weaing</t>
   </si>
 </sst>
 </file>
@@ -3315,6 +3348,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="39" fillId="41" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3326,12 +3365,6 @@
     </xf>
     <xf numFmtId="0" fontId="39" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="44">
@@ -16679,7 +16712,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:K111"/>
+  <dimension ref="A1:K124"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -18067,351 +18100,310 @@
       <c r="K74" s="95"/>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C75" t="s">
+      <c r="A75" s="4" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>2</v>
+      </c>
+      <c r="C76" s="109" t="s">
         <v>18</v>
       </c>
-      <c r="G75" t="s">
+      <c r="G76" t="s">
+        <v>599</v>
+      </c>
+      <c r="H76" s="13">
+        <f>H32*0.035</f>
+        <v>22.803487476595752</v>
+      </c>
+      <c r="I76" t="s">
+        <v>601</v>
+      </c>
+      <c r="K76" s="253" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C77" s="109" t="s">
+        <v>400</v>
+      </c>
+      <c r="G77" t="s">
+        <v>599</v>
+      </c>
+      <c r="H77" s="13">
+        <f>H33*0.03</f>
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C78" s="109" t="s">
+        <v>20</v>
+      </c>
+      <c r="G78" t="s">
+        <v>599</v>
+      </c>
+      <c r="H78" s="13">
+        <f>AVERAGE(H34,H36)*0.03</f>
+        <v>5.6854028249999997</v>
+      </c>
+      <c r="J78" s="93" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C79" s="109" t="s">
+        <v>33</v>
+      </c>
+      <c r="G79" t="s">
+        <v>599</v>
+      </c>
+      <c r="H79" s="13">
+        <f>AVERAGE(H36,H37)*0.03</f>
+        <v>14.026850856000001</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C80" s="109" t="s">
+        <v>34</v>
+      </c>
+      <c r="G80" t="s">
+        <v>599</v>
+      </c>
+      <c r="H80" s="13">
+        <f>AVERAGE(H36,H38)*0.03</f>
+        <v>14.859617133</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C81" s="109" t="s">
+        <v>35</v>
+      </c>
+      <c r="G81" t="s">
+        <v>599</v>
+      </c>
+      <c r="H81" s="13">
+        <f>AVERAGE(H36,H39)*0.03</f>
+        <v>14.95169952</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A83" s="4" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C84" t="s">
+        <v>18</v>
+      </c>
+      <c r="G84" t="s">
         <v>384</v>
       </c>
-      <c r="H75">
+      <c r="H84">
         <v>0.50700000000000001</v>
       </c>
-      <c r="I75" t="s">
+      <c r="I84" t="s">
         <v>385</v>
       </c>
-      <c r="K75" t="s">
+      <c r="K84" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G76" t="s">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G85" t="s">
         <v>384</v>
       </c>
-      <c r="H76">
+      <c r="H85">
         <v>0.47499999999999998</v>
       </c>
-      <c r="I76" t="s">
+      <c r="I85" t="s">
         <v>385</v>
       </c>
-      <c r="K76" t="s">
+      <c r="K85" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C77" t="s">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C86" t="s">
         <v>18</v>
       </c>
-      <c r="G77" t="s">
+      <c r="G86" t="s">
         <v>396</v>
       </c>
-      <c r="H77" s="13">
+      <c r="H86" s="13">
         <v>5</v>
       </c>
-      <c r="I77" t="s">
+      <c r="I86" t="s">
         <v>395</v>
       </c>
-      <c r="K77" t="s">
+      <c r="K86" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>2</v>
       </c>
-      <c r="C78" t="s">
+      <c r="C87" t="s">
         <v>18</v>
       </c>
-      <c r="G78" t="s">
+      <c r="G87" t="s">
         <v>389</v>
       </c>
-      <c r="H78" s="13">
+      <c r="H87" s="13">
         <f>(0.013+0.021+0.038) * 30.4</f>
         <v>2.1888000000000001</v>
       </c>
-      <c r="I78" t="s">
+      <c r="I87" t="s">
         <v>390</v>
       </c>
-      <c r="J78" t="s">
+      <c r="J87" t="s">
         <v>391</v>
       </c>
-      <c r="K78" t="s">
+      <c r="K87" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G79" t="s">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G88" t="s">
         <v>392</v>
       </c>
-      <c r="H79" s="1">
+      <c r="H88" s="1">
         <v>1</v>
       </c>
-      <c r="I79" t="s">
+      <c r="I88" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>2</v>
       </c>
-      <c r="C80" t="s">
+      <c r="C89" t="s">
         <v>18</v>
       </c>
-      <c r="G80" t="s">
+      <c r="G89" t="s">
         <v>392</v>
       </c>
-      <c r="H80" s="1">
+      <c r="H89" s="1">
         <v>1.1100000000000001</v>
       </c>
-      <c r="I80" t="s">
+      <c r="I89" t="s">
         <v>397</v>
       </c>
-      <c r="K80" t="s">
+      <c r="K89" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="C81" t="s">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C90" t="s">
         <v>33</v>
       </c>
-      <c r="G81" t="s">
+      <c r="G90" t="s">
         <v>392</v>
       </c>
-      <c r="H81" s="1">
+      <c r="H90" s="1">
         <v>1.05</v>
       </c>
-      <c r="I81" t="s">
+      <c r="I90" t="s">
         <v>397</v>
       </c>
-      <c r="K81" t="s">
+      <c r="K90" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>2</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C91" t="s">
         <v>34</v>
       </c>
-      <c r="G82" t="s">
+      <c r="G91" t="s">
         <v>392</v>
       </c>
-      <c r="H82" s="1">
+      <c r="H91" s="1">
         <v>1.05</v>
       </c>
-      <c r="I82" t="s">
+      <c r="I91" t="s">
         <v>397</v>
       </c>
-      <c r="K82" t="s">
+      <c r="K91" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G83" t="s">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G92" t="s">
         <v>394</v>
       </c>
-      <c r="H83" s="13">
+      <c r="H92" s="13">
         <v>0</v>
       </c>
-      <c r="I83" t="s">
+      <c r="I92" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>2</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C93" t="s">
         <v>18</v>
       </c>
-      <c r="G84" t="s">
+      <c r="G93" t="s">
         <v>394</v>
       </c>
-      <c r="H84" s="13">
+      <c r="H93" s="13">
         <v>-13.6</v>
       </c>
-      <c r="I84" t="s">
+      <c r="I93" t="s">
         <v>397</v>
       </c>
-      <c r="K84" t="s">
+      <c r="K93" t="s">
         <v>386</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>2</v>
-      </c>
-      <c r="G85" t="s">
-        <v>575</v>
-      </c>
-      <c r="H85" s="2">
-        <v>81</v>
-      </c>
-      <c r="I85" t="s">
-        <v>573</v>
-      </c>
-      <c r="J85" t="s">
-        <v>580</v>
-      </c>
-      <c r="K85" s="253" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G86" t="s">
-        <v>576</v>
-      </c>
-      <c r="H86" s="13">
-        <f>18.8*0.13</f>
-        <v>2.4440000000000004</v>
-      </c>
-      <c r="I86" t="s">
-        <v>572</v>
-      </c>
-      <c r="J86" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H87" s="2"/>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H88" s="13"/>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A89" s="94" t="s">
-        <v>382</v>
-      </c>
-      <c r="B89" s="94"/>
-      <c r="C89" s="95"/>
-      <c r="D89" s="95"/>
-      <c r="E89" s="95"/>
-      <c r="F89" s="95"/>
-      <c r="G89" s="95"/>
-      <c r="H89" s="95"/>
-      <c r="I89" s="95" t="s">
-        <v>310</v>
-      </c>
-      <c r="J89" s="95"/>
-      <c r="K89" s="95"/>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G90" s="158" t="s">
-        <v>309</v>
-      </c>
-      <c r="H90" s="158">
-        <v>0</v>
-      </c>
-      <c r="I90" s="158"/>
-      <c r="J90" s="158" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A91" s="97" t="s">
-        <v>290</v>
-      </c>
-      <c r="B91" s="97"/>
-      <c r="C91" s="98"/>
-      <c r="D91" s="98"/>
-      <c r="E91" s="98"/>
-      <c r="F91" s="98"/>
-      <c r="G91" s="98"/>
-      <c r="H91" s="99"/>
-      <c r="I91" s="98"/>
-      <c r="J91" s="98"/>
-      <c r="K91" s="98"/>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A92" s="81" t="s">
-        <v>63</v>
-      </c>
-      <c r="B92" s="48"/>
-      <c r="C92" s="49"/>
-      <c r="D92" s="49"/>
-      <c r="E92" s="49"/>
-      <c r="F92" s="49"/>
-      <c r="G92" s="49"/>
-      <c r="H92" s="161"/>
-      <c r="I92" s="49"/>
-      <c r="J92" s="49"/>
-      <c r="K92" s="49"/>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A93" s="158" t="s">
-        <v>2</v>
-      </c>
-      <c r="B93" s="158"/>
-      <c r="C93" s="158" t="s">
-        <v>18</v>
-      </c>
-      <c r="G93" s="158" t="s">
-        <v>309</v>
-      </c>
-      <c r="H93" s="158">
-        <v>0</v>
-      </c>
-      <c r="I93" s="158"/>
-      <c r="J93" s="158" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>2</v>
       </c>
-      <c r="C94" t="s">
-        <v>18</v>
-      </c>
-      <c r="D94" t="s">
-        <v>409</v>
-      </c>
       <c r="G94" t="s">
-        <v>309</v>
-      </c>
-      <c r="H94" s="13">
-        <v>45</v>
-      </c>
-      <c r="I94" s="158"/>
-      <c r="J94" s="158"/>
+        <v>575</v>
+      </c>
+      <c r="H94" s="2">
+        <v>81</v>
+      </c>
+      <c r="I94" t="s">
+        <v>573</v>
+      </c>
+      <c r="J94" t="s">
+        <v>580</v>
+      </c>
+      <c r="K94" s="253" t="s">
+        <v>577</v>
+      </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>2</v>
-      </c>
-      <c r="C95" t="s">
-        <v>18</v>
-      </c>
-      <c r="D95" t="s">
-        <v>410</v>
-      </c>
       <c r="G95" t="s">
-        <v>309</v>
+        <v>576</v>
       </c>
       <c r="H95" s="13">
-        <v>12</v>
-      </c>
-      <c r="I95" s="158"/>
-      <c r="J95" s="158"/>
+        <f>18.8*0.13</f>
+        <v>2.4440000000000004</v>
+      </c>
+      <c r="I95" t="s">
+        <v>572</v>
+      </c>
+      <c r="J95" t="s">
+        <v>579</v>
+      </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>2</v>
-      </c>
-      <c r="C96" t="s">
-        <v>18</v>
-      </c>
-      <c r="D96" t="s">
-        <v>398</v>
-      </c>
-      <c r="G96" t="s">
-        <v>309</v>
-      </c>
-      <c r="H96" s="13">
-        <v>6</v>
-      </c>
-      <c r="I96" s="158"/>
-      <c r="J96" s="158"/>
+      <c r="A96" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="H96" s="2"/>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
@@ -18420,145 +18412,151 @@
       <c r="C97" t="s">
         <v>18</v>
       </c>
-      <c r="D97" t="s">
-        <v>371</v>
-      </c>
       <c r="G97" t="s">
-        <v>309</v>
+        <v>594</v>
       </c>
       <c r="H97" s="13">
+        <v>7.6</v>
+      </c>
+      <c r="I97" t="s">
+        <v>595</v>
+      </c>
+      <c r="K97" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A98" s="4"/>
+      <c r="C98" t="s">
         <v>20</v>
       </c>
-      <c r="I97" s="158"/>
-      <c r="J97" s="158"/>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>2</v>
-      </c>
-      <c r="C98" t="s">
-        <v>18</v>
-      </c>
-      <c r="D98" t="s">
-        <v>408</v>
-      </c>
       <c r="G98" t="s">
-        <v>309</v>
+        <v>594</v>
       </c>
       <c r="H98" s="13">
         <v>7</v>
       </c>
+      <c r="I98" t="s">
+        <v>595</v>
+      </c>
+      <c r="J98" t="s">
+        <v>597</v>
+      </c>
+      <c r="K98" t="s">
+        <v>596</v>
+      </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+      <c r="A99" s="4"/>
+      <c r="G99" t="s">
+        <v>594</v>
+      </c>
+      <c r="H99" s="13">
+        <v>6.5</v>
+      </c>
+      <c r="I99" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H100" s="2"/>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H101" s="13"/>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A102" s="94" t="s">
+        <v>382</v>
+      </c>
+      <c r="B102" s="94"/>
+      <c r="C102" s="95"/>
+      <c r="D102" s="95"/>
+      <c r="E102" s="95"/>
+      <c r="F102" s="95"/>
+      <c r="G102" s="95"/>
+      <c r="H102" s="95"/>
+      <c r="I102" s="95" t="s">
+        <v>310</v>
+      </c>
+      <c r="J102" s="95"/>
+      <c r="K102" s="95"/>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G103" s="158" t="s">
+        <v>309</v>
+      </c>
+      <c r="H103" s="158">
+        <v>0</v>
+      </c>
+      <c r="I103" s="158"/>
+      <c r="J103" s="158" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A104" s="97" t="s">
+        <v>290</v>
+      </c>
+      <c r="B104" s="97"/>
+      <c r="C104" s="98"/>
+      <c r="D104" s="98"/>
+      <c r="E104" s="98"/>
+      <c r="F104" s="98"/>
+      <c r="G104" s="98"/>
+      <c r="H104" s="99"/>
+      <c r="I104" s="98"/>
+      <c r="J104" s="98"/>
+      <c r="K104" s="98"/>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A105" s="81" t="s">
+        <v>63</v>
+      </c>
+      <c r="B105" s="48"/>
+      <c r="C105" s="49"/>
+      <c r="D105" s="49"/>
+      <c r="E105" s="49"/>
+      <c r="F105" s="49"/>
+      <c r="G105" s="49"/>
+      <c r="H105" s="161"/>
+      <c r="I105" s="49"/>
+      <c r="J105" s="49"/>
+      <c r="K105" s="49"/>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A106" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="C99" t="s">
+      <c r="B106" s="158"/>
+      <c r="C106" s="158" t="s">
         <v>18</v>
       </c>
-      <c r="D99" t="s">
-        <v>466</v>
-      </c>
-      <c r="G99" t="s">
+      <c r="G106" s="158" t="s">
         <v>309</v>
       </c>
-      <c r="H99" s="13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>2</v>
-      </c>
-      <c r="C100" t="s">
-        <v>18</v>
-      </c>
-      <c r="D100" t="s">
-        <v>403</v>
-      </c>
-      <c r="G100" t="s">
-        <v>309</v>
-      </c>
-      <c r="H100" s="13">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A103" s="81" t="s">
-        <v>448</v>
-      </c>
-      <c r="B103" s="48"/>
-      <c r="C103" s="49"/>
-      <c r="D103" s="49"/>
-      <c r="E103" s="49"/>
-      <c r="F103" s="49"/>
-      <c r="G103" s="49"/>
-      <c r="H103" s="161"/>
-      <c r="I103" s="49"/>
-      <c r="J103" s="49"/>
-      <c r="K103" s="49"/>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A104" s="158" t="s">
-        <v>2</v>
-      </c>
-      <c r="B104" s="158"/>
-      <c r="C104" s="158"/>
-      <c r="G104" s="158" t="s">
-        <v>309</v>
-      </c>
-      <c r="H104" s="158">
+      <c r="H106" s="158">
         <v>0</v>
       </c>
-      <c r="I104" s="158"/>
-      <c r="J104" s="158" t="s">
+      <c r="I106" s="158"/>
+      <c r="J106" s="158" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>2</v>
-      </c>
-      <c r="D105" t="s">
-        <v>409</v>
-      </c>
-      <c r="G105" t="s">
-        <v>309</v>
-      </c>
-      <c r="H105" s="13">
-        <v>0</v>
-      </c>
-      <c r="I105" s="158"/>
-      <c r="J105" s="158"/>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>2</v>
-      </c>
-      <c r="D106" t="s">
-        <v>410</v>
-      </c>
-      <c r="G106" t="s">
-        <v>309</v>
-      </c>
-      <c r="H106" s="13">
-        <v>55</v>
-      </c>
-      <c r="I106" s="158"/>
-      <c r="J106" s="158"/>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>2</v>
       </c>
+      <c r="C107" t="s">
+        <v>18</v>
+      </c>
       <c r="D107" t="s">
-        <v>398</v>
+        <v>409</v>
       </c>
       <c r="G107" t="s">
         <v>309</v>
       </c>
       <c r="H107" s="13">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I107" s="158"/>
       <c r="J107" s="158"/>
@@ -18567,14 +18565,17 @@
       <c r="A108" t="s">
         <v>2</v>
       </c>
+      <c r="C108" t="s">
+        <v>18</v>
+      </c>
       <c r="D108" t="s">
-        <v>371</v>
+        <v>410</v>
       </c>
       <c r="G108" t="s">
         <v>309</v>
       </c>
       <c r="H108" s="13">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I108" s="158"/>
       <c r="J108" s="158"/>
@@ -18583,14 +18584,17 @@
       <c r="A109" t="s">
         <v>2</v>
       </c>
+      <c r="C109" t="s">
+        <v>18</v>
+      </c>
       <c r="D109" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="G109" t="s">
         <v>309</v>
       </c>
       <c r="H109" s="13">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I109" s="158"/>
       <c r="J109" s="158"/>
@@ -18599,14 +18603,17 @@
       <c r="A110" t="s">
         <v>2</v>
       </c>
+      <c r="C110" t="s">
+        <v>18</v>
+      </c>
       <c r="D110" t="s">
-        <v>466</v>
+        <v>371</v>
       </c>
       <c r="G110" t="s">
         <v>309</v>
       </c>
       <c r="H110" s="13">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I110" s="158"/>
       <c r="J110" s="158"/>
@@ -18615,24 +18622,204 @@
       <c r="A111" t="s">
         <v>2</v>
       </c>
+      <c r="C111" t="s">
+        <v>18</v>
+      </c>
       <c r="D111" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="G111" t="s">
         <v>309</v>
       </c>
       <c r="H111" s="13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>2</v>
+      </c>
+      <c r="C112" t="s">
+        <v>18</v>
+      </c>
+      <c r="D112" t="s">
+        <v>466</v>
+      </c>
+      <c r="G112" t="s">
+        <v>309</v>
+      </c>
+      <c r="H112" s="13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>2</v>
+      </c>
+      <c r="C113" t="s">
+        <v>18</v>
+      </c>
+      <c r="D113" t="s">
+        <v>403</v>
+      </c>
+      <c r="G113" t="s">
+        <v>309</v>
+      </c>
+      <c r="H113" s="13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A116" s="81" t="s">
+        <v>448</v>
+      </c>
+      <c r="B116" s="48"/>
+      <c r="C116" s="49"/>
+      <c r="D116" s="49"/>
+      <c r="E116" s="49"/>
+      <c r="F116" s="49"/>
+      <c r="G116" s="49"/>
+      <c r="H116" s="161"/>
+      <c r="I116" s="49"/>
+      <c r="J116" s="49"/>
+      <c r="K116" s="49"/>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A117" s="158" t="s">
+        <v>2</v>
+      </c>
+      <c r="B117" s="158"/>
+      <c r="C117" s="158"/>
+      <c r="G117" s="158" t="s">
+        <v>309</v>
+      </c>
+      <c r="H117" s="158">
         <v>0</v>
       </c>
-      <c r="I111" s="158"/>
-      <c r="J111" s="158"/>
+      <c r="I117" s="158"/>
+      <c r="J117" s="158" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>2</v>
+      </c>
+      <c r="D118" t="s">
+        <v>409</v>
+      </c>
+      <c r="G118" t="s">
+        <v>309</v>
+      </c>
+      <c r="H118" s="13">
+        <v>0</v>
+      </c>
+      <c r="I118" s="158"/>
+      <c r="J118" s="158"/>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>2</v>
+      </c>
+      <c r="D119" t="s">
+        <v>410</v>
+      </c>
+      <c r="G119" t="s">
+        <v>309</v>
+      </c>
+      <c r="H119" s="13">
+        <v>55</v>
+      </c>
+      <c r="I119" s="158"/>
+      <c r="J119" s="158"/>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>2</v>
+      </c>
+      <c r="D120" t="s">
+        <v>398</v>
+      </c>
+      <c r="G120" t="s">
+        <v>309</v>
+      </c>
+      <c r="H120" s="13">
+        <v>40</v>
+      </c>
+      <c r="I120" s="158"/>
+      <c r="J120" s="158"/>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>2</v>
+      </c>
+      <c r="D121" t="s">
+        <v>371</v>
+      </c>
+      <c r="G121" t="s">
+        <v>309</v>
+      </c>
+      <c r="H121" s="13">
+        <v>5</v>
+      </c>
+      <c r="I121" s="158"/>
+      <c r="J121" s="158"/>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>2</v>
+      </c>
+      <c r="D122" t="s">
+        <v>408</v>
+      </c>
+      <c r="G122" t="s">
+        <v>309</v>
+      </c>
+      <c r="H122" s="13">
+        <v>0</v>
+      </c>
+      <c r="I122" s="158"/>
+      <c r="J122" s="158"/>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>2</v>
+      </c>
+      <c r="D123" t="s">
+        <v>466</v>
+      </c>
+      <c r="G123" t="s">
+        <v>309</v>
+      </c>
+      <c r="H123" s="13">
+        <v>0</v>
+      </c>
+      <c r="I123" s="158"/>
+      <c r="J123" s="158"/>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>2</v>
+      </c>
+      <c r="D124" t="s">
+        <v>403</v>
+      </c>
+      <c r="G124" t="s">
+        <v>309</v>
+      </c>
+      <c r="H124" s="13">
+        <v>0</v>
+      </c>
+      <c r="I124" s="158"/>
+      <c r="J124" s="158"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="K85" r:id="rId1"/>
+    <hyperlink ref="K94" r:id="rId1"/>
+    <hyperlink ref="K76" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -24734,49 +24921,49 @@
       </c>
       <c r="AB3" s="198"/>
       <c r="AC3" s="198"/>
-      <c r="AD3" s="268" t="s">
+      <c r="AD3" s="270" t="s">
         <v>508</v>
       </c>
-      <c r="AE3" s="269" t="s">
+      <c r="AE3" s="271" t="s">
         <v>510</v>
       </c>
-      <c r="AF3" s="268" t="s">
+      <c r="AF3" s="270" t="s">
         <v>512</v>
       </c>
-      <c r="AG3" s="269" t="s">
+      <c r="AG3" s="271" t="s">
         <v>514</v>
       </c>
-      <c r="AH3" s="268" t="s">
+      <c r="AH3" s="270" t="s">
         <v>515</v>
       </c>
-      <c r="AI3" s="269" t="s">
+      <c r="AI3" s="271" t="s">
         <v>517</v>
       </c>
-      <c r="AJ3" s="268" t="s">
+      <c r="AJ3" s="270" t="s">
         <v>518</v>
       </c>
-      <c r="AK3" s="269" t="s">
+      <c r="AK3" s="271" t="s">
         <v>519</v>
       </c>
-      <c r="AL3" s="268" t="s">
+      <c r="AL3" s="270" t="s">
         <v>521</v>
       </c>
-      <c r="AM3" s="269" t="s">
+      <c r="AM3" s="271" t="s">
         <v>522</v>
       </c>
-      <c r="AN3" s="268" t="s">
+      <c r="AN3" s="270" t="s">
         <v>542</v>
       </c>
-      <c r="AO3" s="269" t="s">
+      <c r="AO3" s="271" t="s">
         <v>524</v>
       </c>
-      <c r="AP3" s="268" t="s">
+      <c r="AP3" s="270" t="s">
         <v>525</v>
       </c>
-      <c r="AQ3" s="267" t="s">
+      <c r="AQ3" s="269" t="s">
         <v>546</v>
       </c>
-      <c r="AR3" s="266" t="s">
+      <c r="AR3" s="268" t="s">
         <v>541</v>
       </c>
     </row>
@@ -24827,21 +25014,21 @@
       <c r="AA4" s="197"/>
       <c r="AB4" s="198"/>
       <c r="AC4" s="198"/>
-      <c r="AD4" s="268"/>
-      <c r="AE4" s="269"/>
-      <c r="AF4" s="268"/>
-      <c r="AG4" s="269"/>
-      <c r="AH4" s="268"/>
-      <c r="AI4" s="269"/>
-      <c r="AJ4" s="268"/>
-      <c r="AK4" s="269"/>
-      <c r="AL4" s="268"/>
-      <c r="AM4" s="269"/>
-      <c r="AN4" s="268"/>
-      <c r="AO4" s="269"/>
-      <c r="AP4" s="268"/>
-      <c r="AQ4" s="267"/>
-      <c r="AR4" s="266"/>
+      <c r="AD4" s="270"/>
+      <c r="AE4" s="271"/>
+      <c r="AF4" s="270"/>
+      <c r="AG4" s="271"/>
+      <c r="AH4" s="270"/>
+      <c r="AI4" s="271"/>
+      <c r="AJ4" s="270"/>
+      <c r="AK4" s="271"/>
+      <c r="AL4" s="270"/>
+      <c r="AM4" s="271"/>
+      <c r="AN4" s="270"/>
+      <c r="AO4" s="271"/>
+      <c r="AP4" s="270"/>
+      <c r="AQ4" s="269"/>
+      <c r="AR4" s="268"/>
     </row>
     <row r="5" spans="2:44" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="205" t="s">
@@ -24922,21 +25109,21 @@
       <c r="AA5" s="197"/>
       <c r="AB5" s="198"/>
       <c r="AC5" s="198"/>
-      <c r="AD5" s="268"/>
-      <c r="AE5" s="269"/>
-      <c r="AF5" s="268"/>
-      <c r="AG5" s="269"/>
-      <c r="AH5" s="268"/>
-      <c r="AI5" s="269"/>
-      <c r="AJ5" s="268"/>
-      <c r="AK5" s="269"/>
-      <c r="AL5" s="268"/>
-      <c r="AM5" s="269"/>
-      <c r="AN5" s="268"/>
-      <c r="AO5" s="269"/>
-      <c r="AP5" s="268"/>
-      <c r="AQ5" s="267"/>
-      <c r="AR5" s="266" t="s">
+      <c r="AD5" s="270"/>
+      <c r="AE5" s="271"/>
+      <c r="AF5" s="270"/>
+      <c r="AG5" s="271"/>
+      <c r="AH5" s="270"/>
+      <c r="AI5" s="271"/>
+      <c r="AJ5" s="270"/>
+      <c r="AK5" s="271"/>
+      <c r="AL5" s="270"/>
+      <c r="AM5" s="271"/>
+      <c r="AN5" s="270"/>
+      <c r="AO5" s="271"/>
+      <c r="AP5" s="270"/>
+      <c r="AQ5" s="269"/>
+      <c r="AR5" s="268" t="s">
         <v>540</v>
       </c>
     </row>
@@ -26371,23 +26558,23 @@
       <c r="N23" s="167"/>
       <c r="O23" s="167"/>
       <c r="P23" s="167"/>
-      <c r="Q23" s="271" t="s">
+      <c r="Q23" s="267" t="s">
         <v>560</v>
       </c>
-      <c r="R23" s="271" t="s">
+      <c r="R23" s="267" t="s">
         <v>561</v>
       </c>
-      <c r="S23" s="271" t="s">
+      <c r="S23" s="267" t="s">
         <v>548</v>
       </c>
-      <c r="T23" s="270" t="s">
+      <c r="T23" s="266" t="s">
         <v>290</v>
       </c>
-      <c r="U23" s="270"/>
-      <c r="V23" s="270" t="s">
+      <c r="U23" s="266"/>
+      <c r="V23" s="266" t="s">
         <v>291</v>
       </c>
-      <c r="W23" s="270"/>
+      <c r="W23" s="266"/>
       <c r="X23" s="166" t="s">
         <v>453</v>
       </c>
@@ -26412,9 +26599,9 @@
       <c r="P24" s="168" t="s">
         <v>454</v>
       </c>
-      <c r="Q24" s="271"/>
-      <c r="R24" s="271"/>
-      <c r="S24" s="271"/>
+      <c r="Q24" s="267"/>
+      <c r="R24" s="267"/>
+      <c r="S24" s="267"/>
       <c r="T24" s="240" t="s">
         <v>454</v>
       </c>
@@ -33211,11 +33398,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="V23:W23"/>
-    <mergeCell ref="T23:U23"/>
-    <mergeCell ref="Q23:Q24"/>
-    <mergeCell ref="R23:R24"/>
-    <mergeCell ref="S23:S24"/>
     <mergeCell ref="AR3:AR5"/>
     <mergeCell ref="AQ3:AQ5"/>
     <mergeCell ref="AD3:AD5"/>
@@ -33231,6 +33413,11 @@
     <mergeCell ref="AN3:AN5"/>
     <mergeCell ref="AO3:AO5"/>
     <mergeCell ref="AP3:AP5"/>
+    <mergeCell ref="V23:W23"/>
+    <mergeCell ref="T23:U23"/>
+    <mergeCell ref="Q23:Q24"/>
+    <mergeCell ref="R23:R24"/>
+    <mergeCell ref="S23:S24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added calc of min/max feed PBV requirements for cattle + parameters in mini dataset
</commit_message>
<xml_diff>
--- a/mini/data/default/CattleHerd.xlsx
+++ b/mini/data/default/CattleHerd.xlsx
@@ -144,7 +144,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2401" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2456" uniqueCount="611">
   <si>
     <t>value</t>
   </si>
@@ -1955,6 +1955,30 @@
   </si>
   <si>
     <t>handle pre weaing</t>
+  </si>
+  <si>
+    <t>Protein (PBV)</t>
+  </si>
+  <si>
+    <t>max_PBV</t>
+  </si>
+  <si>
+    <t>g PBV/head/day</t>
+  </si>
+  <si>
+    <t>min_PBV</t>
+  </si>
+  <si>
+    <t>max_PBV_per_ME</t>
+  </si>
+  <si>
+    <t>g PBV/MJ ME</t>
+  </si>
+  <si>
+    <t>min_PBV_per_ME</t>
+  </si>
+  <si>
+    <t>Same as growing animals?</t>
   </si>
 </sst>
 </file>
@@ -2925,7 +2949,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="272">
+  <cellXfs count="273">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3348,12 +3372,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="39" fillId="41" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3366,6 +3384,13 @@
     <xf numFmtId="0" fontId="39" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -16712,7 +16737,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:K124"/>
+  <dimension ref="A1:K143"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -18459,359 +18484,611 @@
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H100" s="2"/>
+      <c r="A100" s="4"/>
+      <c r="H100" s="13"/>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="H101" s="13"/>
+      <c r="A101" s="4" t="s">
+        <v>603</v>
+      </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A102" s="94" t="s">
-        <v>382</v>
-      </c>
-      <c r="B102" s="94"/>
-      <c r="C102" s="95"/>
-      <c r="D102" s="95"/>
-      <c r="E102" s="95"/>
-      <c r="F102" s="95"/>
-      <c r="G102" s="95"/>
-      <c r="H102" s="95"/>
-      <c r="I102" s="95" t="s">
-        <v>310</v>
-      </c>
-      <c r="J102" s="95"/>
-      <c r="K102" s="95"/>
+      <c r="G102" s="158" t="s">
+        <v>604</v>
+      </c>
+      <c r="H102" s="272">
+        <v>0</v>
+      </c>
+      <c r="I102" s="158" t="s">
+        <v>605</v>
+      </c>
+      <c r="J102" s="158" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G103" s="158" t="s">
-        <v>309</v>
-      </c>
-      <c r="H103" s="158">
+        <v>606</v>
+      </c>
+      <c r="H103" s="272">
         <v>0</v>
       </c>
-      <c r="I103" s="158"/>
+      <c r="I103" s="158" t="s">
+        <v>605</v>
+      </c>
       <c r="J103" s="158" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A104" s="97" t="s">
-        <v>290</v>
-      </c>
-      <c r="B104" s="97"/>
-      <c r="C104" s="98"/>
-      <c r="D104" s="98"/>
-      <c r="E104" s="98"/>
-      <c r="F104" s="98"/>
-      <c r="G104" s="98"/>
-      <c r="H104" s="99"/>
-      <c r="I104" s="98"/>
-      <c r="J104" s="98"/>
-      <c r="K104" s="98"/>
+      <c r="G104" s="158" t="s">
+        <v>607</v>
+      </c>
+      <c r="H104" s="272">
+        <v>0</v>
+      </c>
+      <c r="I104" s="158" t="s">
+        <v>608</v>
+      </c>
+      <c r="J104" s="158" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A105" s="81" t="s">
-        <v>63</v>
-      </c>
-      <c r="B105" s="48"/>
-      <c r="C105" s="49"/>
-      <c r="D105" s="49"/>
-      <c r="E105" s="49"/>
-      <c r="F105" s="49"/>
-      <c r="G105" s="49"/>
-      <c r="H105" s="161"/>
-      <c r="I105" s="49"/>
-      <c r="J105" s="49"/>
-      <c r="K105" s="49"/>
+      <c r="G105" s="158" t="s">
+        <v>609</v>
+      </c>
+      <c r="H105" s="272">
+        <v>0</v>
+      </c>
+      <c r="I105" s="158" t="s">
+        <v>608</v>
+      </c>
+      <c r="J105" s="158" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A106" s="158" t="s">
-        <v>2</v>
-      </c>
-      <c r="B106" s="158"/>
-      <c r="C106" s="158" t="s">
-        <v>18</v>
-      </c>
-      <c r="G106" s="158" t="s">
-        <v>309</v>
-      </c>
-      <c r="H106" s="158">
-        <v>0</v>
-      </c>
-      <c r="I106" s="158"/>
-      <c r="J106" s="158" t="s">
-        <v>399</v>
-      </c>
+      <c r="H106" s="2"/>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>2</v>
-      </c>
       <c r="C107" t="s">
         <v>18</v>
       </c>
-      <c r="D107" t="s">
-        <v>409</v>
-      </c>
       <c r="G107" t="s">
-        <v>309</v>
-      </c>
-      <c r="H107" s="13">
-        <v>45</v>
-      </c>
-      <c r="I107" s="158"/>
-      <c r="J107" s="158"/>
+        <v>604</v>
+      </c>
+      <c r="H107" s="2">
+        <v>300</v>
+      </c>
+      <c r="I107" t="s">
+        <v>605</v>
+      </c>
+      <c r="K107" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>2</v>
-      </c>
       <c r="C108" t="s">
         <v>18</v>
       </c>
-      <c r="D108" t="s">
+      <c r="G108" t="s">
+        <v>606</v>
+      </c>
+      <c r="H108" s="2">
+        <v>0</v>
+      </c>
+      <c r="I108" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C110" s="109" t="s">
+        <v>400</v>
+      </c>
+      <c r="G110" t="s">
+        <v>607</v>
+      </c>
+      <c r="H110" s="2">
+        <v>4</v>
+      </c>
+      <c r="I110" t="s">
+        <v>608</v>
+      </c>
+      <c r="J110" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C111" s="109" t="s">
+        <v>400</v>
+      </c>
+      <c r="G111" t="s">
+        <v>609</v>
+      </c>
+      <c r="H111" s="2">
+        <v>-2</v>
+      </c>
+      <c r="I111" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C112" s="109" t="s">
+        <v>20</v>
+      </c>
+      <c r="G112" t="s">
+        <v>607</v>
+      </c>
+      <c r="H112" s="2">
+        <v>4</v>
+      </c>
+      <c r="I112" t="s">
+        <v>608</v>
+      </c>
+      <c r="K112" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C113" s="109" t="s">
+        <v>20</v>
+      </c>
+      <c r="G113" t="s">
+        <v>609</v>
+      </c>
+      <c r="H113" s="2">
+        <v>-2</v>
+      </c>
+      <c r="I113" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C114" s="109" t="s">
+        <v>33</v>
+      </c>
+      <c r="G114" t="s">
+        <v>607</v>
+      </c>
+      <c r="H114" s="2">
+        <v>4</v>
+      </c>
+      <c r="I114" t="s">
+        <v>608</v>
+      </c>
+      <c r="K114" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C115" s="109" t="s">
+        <v>33</v>
+      </c>
+      <c r="G115" t="s">
+        <v>609</v>
+      </c>
+      <c r="H115" s="2">
+        <v>-2</v>
+      </c>
+      <c r="I115" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C116" s="109" t="s">
+        <v>34</v>
+      </c>
+      <c r="G116" t="s">
+        <v>607</v>
+      </c>
+      <c r="H116" s="2">
+        <v>4</v>
+      </c>
+      <c r="I116" t="s">
+        <v>608</v>
+      </c>
+      <c r="K116" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C117" s="109" t="s">
+        <v>34</v>
+      </c>
+      <c r="G117" t="s">
+        <v>609</v>
+      </c>
+      <c r="H117" s="2">
+        <v>-2</v>
+      </c>
+      <c r="I117" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C118" s="109" t="s">
+        <v>35</v>
+      </c>
+      <c r="G118" t="s">
+        <v>607</v>
+      </c>
+      <c r="H118" s="2">
+        <v>4</v>
+      </c>
+      <c r="I118" t="s">
+        <v>608</v>
+      </c>
+      <c r="K118" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C119" s="109" t="s">
+        <v>35</v>
+      </c>
+      <c r="G119" t="s">
+        <v>609</v>
+      </c>
+      <c r="H119" s="2">
+        <v>-2</v>
+      </c>
+      <c r="I119" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C120" s="109"/>
+      <c r="H120" s="2"/>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A121" s="94" t="s">
+        <v>382</v>
+      </c>
+      <c r="B121" s="94"/>
+      <c r="C121" s="95"/>
+      <c r="D121" s="95"/>
+      <c r="E121" s="95"/>
+      <c r="F121" s="95"/>
+      <c r="G121" s="95"/>
+      <c r="H121" s="95"/>
+      <c r="I121" s="95" t="s">
+        <v>310</v>
+      </c>
+      <c r="J121" s="95"/>
+      <c r="K121" s="95"/>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G122" s="158" t="s">
+        <v>309</v>
+      </c>
+      <c r="H122" s="158">
+        <v>0</v>
+      </c>
+      <c r="I122" s="158"/>
+      <c r="J122" s="158" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A123" s="97" t="s">
+        <v>290</v>
+      </c>
+      <c r="B123" s="97"/>
+      <c r="C123" s="98"/>
+      <c r="D123" s="98"/>
+      <c r="E123" s="98"/>
+      <c r="F123" s="98"/>
+      <c r="G123" s="98"/>
+      <c r="H123" s="99"/>
+      <c r="I123" s="98"/>
+      <c r="J123" s="98"/>
+      <c r="K123" s="98"/>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A124" s="81" t="s">
+        <v>63</v>
+      </c>
+      <c r="B124" s="48"/>
+      <c r="C124" s="49"/>
+      <c r="D124" s="49"/>
+      <c r="E124" s="49"/>
+      <c r="F124" s="49"/>
+      <c r="G124" s="49"/>
+      <c r="H124" s="161"/>
+      <c r="I124" s="49"/>
+      <c r="J124" s="49"/>
+      <c r="K124" s="49"/>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A125" s="158" t="s">
+        <v>2</v>
+      </c>
+      <c r="B125" s="158"/>
+      <c r="C125" s="158" t="s">
+        <v>18</v>
+      </c>
+      <c r="G125" s="158" t="s">
+        <v>309</v>
+      </c>
+      <c r="H125" s="158">
+        <v>0</v>
+      </c>
+      <c r="I125" s="158"/>
+      <c r="J125" s="158" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>2</v>
+      </c>
+      <c r="C126" t="s">
+        <v>18</v>
+      </c>
+      <c r="D126" t="s">
+        <v>409</v>
+      </c>
+      <c r="G126" t="s">
+        <v>309</v>
+      </c>
+      <c r="H126" s="13">
+        <v>45</v>
+      </c>
+      <c r="I126" s="158"/>
+      <c r="J126" s="158"/>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>2</v>
+      </c>
+      <c r="C127" t="s">
+        <v>18</v>
+      </c>
+      <c r="D127" t="s">
         <v>410</v>
       </c>
-      <c r="G108" t="s">
+      <c r="G127" t="s">
         <v>309</v>
       </c>
-      <c r="H108" s="13">
+      <c r="H127" s="13">
         <v>12</v>
       </c>
-      <c r="I108" s="158"/>
-      <c r="J108" s="158"/>
-    </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+      <c r="I127" s="158"/>
+      <c r="J127" s="158"/>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
         <v>2</v>
       </c>
-      <c r="C109" t="s">
+      <c r="C128" t="s">
         <v>18</v>
       </c>
-      <c r="D109" t="s">
+      <c r="D128" t="s">
         <v>398</v>
       </c>
-      <c r="G109" t="s">
+      <c r="G128" t="s">
         <v>309</v>
       </c>
-      <c r="H109" s="13">
+      <c r="H128" s="13">
         <v>6</v>
       </c>
-      <c r="I109" s="158"/>
-      <c r="J109" s="158"/>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
+      <c r="I128" s="158"/>
+      <c r="J128" s="158"/>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
         <v>2</v>
       </c>
-      <c r="C110" t="s">
+      <c r="C129" t="s">
         <v>18</v>
       </c>
-      <c r="D110" t="s">
+      <c r="D129" t="s">
         <v>371</v>
       </c>
-      <c r="G110" t="s">
+      <c r="G129" t="s">
         <v>309</v>
       </c>
-      <c r="H110" s="13">
+      <c r="H129" s="13">
         <v>20</v>
       </c>
-      <c r="I110" s="158"/>
-      <c r="J110" s="158"/>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
+      <c r="I129" s="158"/>
+      <c r="J129" s="158"/>
+    </row>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
         <v>2</v>
       </c>
-      <c r="C111" t="s">
+      <c r="C130" t="s">
         <v>18</v>
       </c>
-      <c r="D111" t="s">
+      <c r="D130" t="s">
         <v>408</v>
       </c>
-      <c r="G111" t="s">
+      <c r="G130" t="s">
         <v>309</v>
       </c>
-      <c r="H111" s="13">
+      <c r="H130" s="13">
         <v>7</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
         <v>2</v>
       </c>
-      <c r="C112" t="s">
+      <c r="C131" t="s">
         <v>18</v>
       </c>
-      <c r="D112" t="s">
+      <c r="D131" t="s">
         <v>466</v>
       </c>
-      <c r="G112" t="s">
+      <c r="G131" t="s">
         <v>309</v>
       </c>
-      <c r="H112" s="13">
+      <c r="H131" s="13">
         <v>3</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
         <v>2</v>
       </c>
-      <c r="C113" t="s">
+      <c r="C132" t="s">
         <v>18</v>
       </c>
-      <c r="D113" t="s">
+      <c r="D132" t="s">
         <v>403</v>
       </c>
-      <c r="G113" t="s">
+      <c r="G132" t="s">
         <v>309</v>
       </c>
-      <c r="H113" s="13">
+      <c r="H132" s="13">
         <v>7</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A116" s="81" t="s">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A135" s="81" t="s">
         <v>448</v>
       </c>
-      <c r="B116" s="48"/>
-      <c r="C116" s="49"/>
-      <c r="D116" s="49"/>
-      <c r="E116" s="49"/>
-      <c r="F116" s="49"/>
-      <c r="G116" s="49"/>
-      <c r="H116" s="161"/>
-      <c r="I116" s="49"/>
-      <c r="J116" s="49"/>
-      <c r="K116" s="49"/>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A117" s="158" t="s">
+      <c r="B135" s="48"/>
+      <c r="C135" s="49"/>
+      <c r="D135" s="49"/>
+      <c r="E135" s="49"/>
+      <c r="F135" s="49"/>
+      <c r="G135" s="49"/>
+      <c r="H135" s="161"/>
+      <c r="I135" s="49"/>
+      <c r="J135" s="49"/>
+      <c r="K135" s="49"/>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A136" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="B117" s="158"/>
-      <c r="C117" s="158"/>
-      <c r="G117" s="158" t="s">
+      <c r="B136" s="158"/>
+      <c r="C136" s="158"/>
+      <c r="G136" s="158" t="s">
         <v>309</v>
       </c>
-      <c r="H117" s="158">
+      <c r="H136" s="158">
         <v>0</v>
       </c>
-      <c r="I117" s="158"/>
-      <c r="J117" s="158" t="s">
+      <c r="I136" s="158"/>
+      <c r="J136" s="158" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
         <v>2</v>
       </c>
-      <c r="D118" t="s">
+      <c r="D137" t="s">
         <v>409</v>
       </c>
-      <c r="G118" t="s">
+      <c r="G137" t="s">
         <v>309</v>
       </c>
-      <c r="H118" s="13">
+      <c r="H137" s="13">
         <v>0</v>
       </c>
-      <c r="I118" s="158"/>
-      <c r="J118" s="158"/>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
+      <c r="I137" s="158"/>
+      <c r="J137" s="158"/>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
         <v>2</v>
       </c>
-      <c r="D119" t="s">
+      <c r="D138" t="s">
         <v>410</v>
       </c>
-      <c r="G119" t="s">
+      <c r="G138" t="s">
         <v>309</v>
       </c>
-      <c r="H119" s="13">
+      <c r="H138" s="13">
         <v>55</v>
       </c>
-      <c r="I119" s="158"/>
-      <c r="J119" s="158"/>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
+      <c r="I138" s="158"/>
+      <c r="J138" s="158"/>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
         <v>2</v>
       </c>
-      <c r="D120" t="s">
+      <c r="D139" t="s">
         <v>398</v>
       </c>
-      <c r="G120" t="s">
+      <c r="G139" t="s">
         <v>309</v>
       </c>
-      <c r="H120" s="13">
+      <c r="H139" s="13">
         <v>40</v>
       </c>
-      <c r="I120" s="158"/>
-      <c r="J120" s="158"/>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
+      <c r="I139" s="158"/>
+      <c r="J139" s="158"/>
+    </row>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
         <v>2</v>
       </c>
-      <c r="D121" t="s">
+      <c r="D140" t="s">
         <v>371</v>
       </c>
-      <c r="G121" t="s">
+      <c r="G140" t="s">
         <v>309</v>
       </c>
-      <c r="H121" s="13">
+      <c r="H140" s="13">
         <v>5</v>
       </c>
-      <c r="I121" s="158"/>
-      <c r="J121" s="158"/>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
+      <c r="I140" s="158"/>
+      <c r="J140" s="158"/>
+    </row>
+    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
         <v>2</v>
       </c>
-      <c r="D122" t="s">
+      <c r="D141" t="s">
         <v>408</v>
       </c>
-      <c r="G122" t="s">
+      <c r="G141" t="s">
         <v>309</v>
       </c>
-      <c r="H122" s="13">
+      <c r="H141" s="13">
         <v>0</v>
       </c>
-      <c r="I122" s="158"/>
-      <c r="J122" s="158"/>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
+      <c r="I141" s="158"/>
+      <c r="J141" s="158"/>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
         <v>2</v>
       </c>
-      <c r="D123" t="s">
+      <c r="D142" t="s">
         <v>466</v>
       </c>
-      <c r="G123" t="s">
+      <c r="G142" t="s">
         <v>309</v>
       </c>
-      <c r="H123" s="13">
+      <c r="H142" s="13">
         <v>0</v>
       </c>
-      <c r="I123" s="158"/>
-      <c r="J123" s="158"/>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
+      <c r="I142" s="158"/>
+      <c r="J142" s="158"/>
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
         <v>2</v>
       </c>
-      <c r="D124" t="s">
+      <c r="D143" t="s">
         <v>403</v>
       </c>
-      <c r="G124" t="s">
+      <c r="G143" t="s">
         <v>309</v>
       </c>
-      <c r="H124" s="13">
+      <c r="H143" s="13">
         <v>0</v>
       </c>
-      <c r="I124" s="158"/>
-      <c r="J124" s="158"/>
+      <c r="I143" s="158"/>
+      <c r="J143" s="158"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -24921,49 +25198,49 @@
       </c>
       <c r="AB3" s="198"/>
       <c r="AC3" s="198"/>
-      <c r="AD3" s="270" t="s">
+      <c r="AD3" s="268" t="s">
         <v>508</v>
       </c>
-      <c r="AE3" s="271" t="s">
+      <c r="AE3" s="269" t="s">
         <v>510</v>
       </c>
-      <c r="AF3" s="270" t="s">
+      <c r="AF3" s="268" t="s">
         <v>512</v>
       </c>
-      <c r="AG3" s="271" t="s">
+      <c r="AG3" s="269" t="s">
         <v>514</v>
       </c>
-      <c r="AH3" s="270" t="s">
+      <c r="AH3" s="268" t="s">
         <v>515</v>
       </c>
-      <c r="AI3" s="271" t="s">
+      <c r="AI3" s="269" t="s">
         <v>517</v>
       </c>
-      <c r="AJ3" s="270" t="s">
+      <c r="AJ3" s="268" t="s">
         <v>518</v>
       </c>
-      <c r="AK3" s="271" t="s">
+      <c r="AK3" s="269" t="s">
         <v>519</v>
       </c>
-      <c r="AL3" s="270" t="s">
+      <c r="AL3" s="268" t="s">
         <v>521</v>
       </c>
-      <c r="AM3" s="271" t="s">
+      <c r="AM3" s="269" t="s">
         <v>522</v>
       </c>
-      <c r="AN3" s="270" t="s">
+      <c r="AN3" s="268" t="s">
         <v>542</v>
       </c>
-      <c r="AO3" s="271" t="s">
+      <c r="AO3" s="269" t="s">
         <v>524</v>
       </c>
-      <c r="AP3" s="270" t="s">
+      <c r="AP3" s="268" t="s">
         <v>525</v>
       </c>
-      <c r="AQ3" s="269" t="s">
+      <c r="AQ3" s="267" t="s">
         <v>546</v>
       </c>
-      <c r="AR3" s="268" t="s">
+      <c r="AR3" s="266" t="s">
         <v>541</v>
       </c>
     </row>
@@ -25014,21 +25291,21 @@
       <c r="AA4" s="197"/>
       <c r="AB4" s="198"/>
       <c r="AC4" s="198"/>
-      <c r="AD4" s="270"/>
-      <c r="AE4" s="271"/>
-      <c r="AF4" s="270"/>
-      <c r="AG4" s="271"/>
-      <c r="AH4" s="270"/>
-      <c r="AI4" s="271"/>
-      <c r="AJ4" s="270"/>
-      <c r="AK4" s="271"/>
-      <c r="AL4" s="270"/>
-      <c r="AM4" s="271"/>
-      <c r="AN4" s="270"/>
-      <c r="AO4" s="271"/>
-      <c r="AP4" s="270"/>
-      <c r="AQ4" s="269"/>
-      <c r="AR4" s="268"/>
+      <c r="AD4" s="268"/>
+      <c r="AE4" s="269"/>
+      <c r="AF4" s="268"/>
+      <c r="AG4" s="269"/>
+      <c r="AH4" s="268"/>
+      <c r="AI4" s="269"/>
+      <c r="AJ4" s="268"/>
+      <c r="AK4" s="269"/>
+      <c r="AL4" s="268"/>
+      <c r="AM4" s="269"/>
+      <c r="AN4" s="268"/>
+      <c r="AO4" s="269"/>
+      <c r="AP4" s="268"/>
+      <c r="AQ4" s="267"/>
+      <c r="AR4" s="266"/>
     </row>
     <row r="5" spans="2:44" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="205" t="s">
@@ -25109,21 +25386,21 @@
       <c r="AA5" s="197"/>
       <c r="AB5" s="198"/>
       <c r="AC5" s="198"/>
-      <c r="AD5" s="270"/>
-      <c r="AE5" s="271"/>
-      <c r="AF5" s="270"/>
-      <c r="AG5" s="271"/>
-      <c r="AH5" s="270"/>
-      <c r="AI5" s="271"/>
-      <c r="AJ5" s="270"/>
-      <c r="AK5" s="271"/>
-      <c r="AL5" s="270"/>
-      <c r="AM5" s="271"/>
-      <c r="AN5" s="270"/>
-      <c r="AO5" s="271"/>
-      <c r="AP5" s="270"/>
-      <c r="AQ5" s="269"/>
-      <c r="AR5" s="268" t="s">
+      <c r="AD5" s="268"/>
+      <c r="AE5" s="269"/>
+      <c r="AF5" s="268"/>
+      <c r="AG5" s="269"/>
+      <c r="AH5" s="268"/>
+      <c r="AI5" s="269"/>
+      <c r="AJ5" s="268"/>
+      <c r="AK5" s="269"/>
+      <c r="AL5" s="268"/>
+      <c r="AM5" s="269"/>
+      <c r="AN5" s="268"/>
+      <c r="AO5" s="269"/>
+      <c r="AP5" s="268"/>
+      <c r="AQ5" s="267"/>
+      <c r="AR5" s="266" t="s">
         <v>540</v>
       </c>
     </row>
@@ -26558,23 +26835,23 @@
       <c r="N23" s="167"/>
       <c r="O23" s="167"/>
       <c r="P23" s="167"/>
-      <c r="Q23" s="267" t="s">
+      <c r="Q23" s="271" t="s">
         <v>560</v>
       </c>
-      <c r="R23" s="267" t="s">
+      <c r="R23" s="271" t="s">
         <v>561</v>
       </c>
-      <c r="S23" s="267" t="s">
+      <c r="S23" s="271" t="s">
         <v>548</v>
       </c>
-      <c r="T23" s="266" t="s">
+      <c r="T23" s="270" t="s">
         <v>290</v>
       </c>
-      <c r="U23" s="266"/>
-      <c r="V23" s="266" t="s">
+      <c r="U23" s="270"/>
+      <c r="V23" s="270" t="s">
         <v>291</v>
       </c>
-      <c r="W23" s="266"/>
+      <c r="W23" s="270"/>
       <c r="X23" s="166" t="s">
         <v>453</v>
       </c>
@@ -26599,9 +26876,9 @@
       <c r="P24" s="168" t="s">
         <v>454</v>
       </c>
-      <c r="Q24" s="267"/>
-      <c r="R24" s="267"/>
-      <c r="S24" s="267"/>
+      <c r="Q24" s="271"/>
+      <c r="R24" s="271"/>
+      <c r="S24" s="271"/>
       <c r="T24" s="240" t="s">
         <v>454</v>
       </c>
@@ -33398,6 +33675,11 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="V23:W23"/>
+    <mergeCell ref="T23:U23"/>
+    <mergeCell ref="Q23:Q24"/>
+    <mergeCell ref="R23:R24"/>
+    <mergeCell ref="S23:S24"/>
     <mergeCell ref="AR3:AR5"/>
     <mergeCell ref="AQ3:AQ5"/>
     <mergeCell ref="AD3:AD5"/>
@@ -33413,11 +33695,6 @@
     <mergeCell ref="AN3:AN5"/>
     <mergeCell ref="AO3:AO5"/>
     <mergeCell ref="AP3:AP5"/>
-    <mergeCell ref="V23:W23"/>
-    <mergeCell ref="T23:U23"/>
-    <mergeCell ref="Q23:Q24"/>
-    <mergeCell ref="R23:R24"/>
-    <mergeCell ref="S23:S24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added feed requirement data_attr for shares of DM + fat constr. for cattle
</commit_message>
<xml_diff>
--- a/mini/data/default/CattleHerd.xlsx
+++ b/mini/data/default/CattleHerd.xlsx
@@ -144,7 +144,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2456" uniqueCount="611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2460" uniqueCount="613">
   <si>
     <t>value</t>
   </si>
@@ -1979,6 +1979,12 @@
   </si>
   <si>
     <t>Same as growing animals?</t>
+  </si>
+  <si>
+    <t>max_fat</t>
+  </si>
+  <si>
+    <t>Spörndly (2003)</t>
   </si>
 </sst>
 </file>
@@ -3372,6 +3378,13 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="39" fillId="41" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3384,13 +3397,6 @@
     <xf numFmtId="0" fontId="39" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -16737,7 +16743,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:K143"/>
+  <dimension ref="A1:K146"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -18496,7 +18502,7 @@
       <c r="G102" s="158" t="s">
         <v>604</v>
       </c>
-      <c r="H102" s="272">
+      <c r="H102" s="266">
         <v>0</v>
       </c>
       <c r="I102" s="158" t="s">
@@ -18510,7 +18516,7 @@
       <c r="G103" s="158" t="s">
         <v>606</v>
       </c>
-      <c r="H103" s="272">
+      <c r="H103" s="266">
         <v>0</v>
       </c>
       <c r="I103" s="158" t="s">
@@ -18524,7 +18530,7 @@
       <c r="G104" s="158" t="s">
         <v>607</v>
       </c>
-      <c r="H104" s="272">
+      <c r="H104" s="266">
         <v>0</v>
       </c>
       <c r="I104" s="158" t="s">
@@ -18538,7 +18544,7 @@
       <c r="G105" s="158" t="s">
         <v>609</v>
       </c>
-      <c r="H105" s="272">
+      <c r="H105" s="266">
         <v>0</v>
       </c>
       <c r="I105" s="158" t="s">
@@ -18742,72 +18748,50 @@
       <c r="H120" s="2"/>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A121" s="94" t="s">
+      <c r="A121" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="C121" s="109"/>
+      <c r="H121" s="2"/>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A122" s="4"/>
+      <c r="C122" s="109"/>
+      <c r="G122" t="s">
+        <v>611</v>
+      </c>
+      <c r="H122" s="2">
+        <v>5</v>
+      </c>
+      <c r="I122" t="s">
+        <v>310</v>
+      </c>
+      <c r="K122" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C123" s="109"/>
+      <c r="H123" s="2"/>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A124" s="94" t="s">
         <v>382</v>
       </c>
-      <c r="B121" s="94"/>
-      <c r="C121" s="95"/>
-      <c r="D121" s="95"/>
-      <c r="E121" s="95"/>
-      <c r="F121" s="95"/>
-      <c r="G121" s="95"/>
-      <c r="H121" s="95"/>
-      <c r="I121" s="95" t="s">
+      <c r="B124" s="94"/>
+      <c r="C124" s="95"/>
+      <c r="D124" s="95"/>
+      <c r="E124" s="95"/>
+      <c r="F124" s="95"/>
+      <c r="G124" s="95"/>
+      <c r="H124" s="95"/>
+      <c r="I124" s="95" t="s">
         <v>310</v>
       </c>
-      <c r="J121" s="95"/>
-      <c r="K121" s="95"/>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G122" s="158" t="s">
-        <v>309</v>
-      </c>
-      <c r="H122" s="158">
-        <v>0</v>
-      </c>
-      <c r="I122" s="158"/>
-      <c r="J122" s="158" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A123" s="97" t="s">
-        <v>290</v>
-      </c>
-      <c r="B123" s="97"/>
-      <c r="C123" s="98"/>
-      <c r="D123" s="98"/>
-      <c r="E123" s="98"/>
-      <c r="F123" s="98"/>
-      <c r="G123" s="98"/>
-      <c r="H123" s="99"/>
-      <c r="I123" s="98"/>
-      <c r="J123" s="98"/>
-      <c r="K123" s="98"/>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A124" s="81" t="s">
-        <v>63</v>
-      </c>
-      <c r="B124" s="48"/>
-      <c r="C124" s="49"/>
-      <c r="D124" s="49"/>
-      <c r="E124" s="49"/>
-      <c r="F124" s="49"/>
-      <c r="G124" s="49"/>
-      <c r="H124" s="161"/>
-      <c r="I124" s="49"/>
-      <c r="J124" s="49"/>
-      <c r="K124" s="49"/>
+      <c r="J124" s="95"/>
+      <c r="K124" s="95"/>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A125" s="158" t="s">
-        <v>2</v>
-      </c>
-      <c r="B125" s="158"/>
-      <c r="C125" s="158" t="s">
-        <v>18</v>
-      </c>
       <c r="G125" s="158" t="s">
         <v>309</v>
       </c>
@@ -18820,61 +18804,53 @@
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
+      <c r="A126" s="97" t="s">
+        <v>290</v>
+      </c>
+      <c r="B126" s="97"/>
+      <c r="C126" s="98"/>
+      <c r="D126" s="98"/>
+      <c r="E126" s="98"/>
+      <c r="F126" s="98"/>
+      <c r="G126" s="98"/>
+      <c r="H126" s="99"/>
+      <c r="I126" s="98"/>
+      <c r="J126" s="98"/>
+      <c r="K126" s="98"/>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A127" s="81" t="s">
+        <v>63</v>
+      </c>
+      <c r="B127" s="48"/>
+      <c r="C127" s="49"/>
+      <c r="D127" s="49"/>
+      <c r="E127" s="49"/>
+      <c r="F127" s="49"/>
+      <c r="G127" s="49"/>
+      <c r="H127" s="161"/>
+      <c r="I127" s="49"/>
+      <c r="J127" s="49"/>
+      <c r="K127" s="49"/>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A128" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="C126" t="s">
+      <c r="B128" s="158"/>
+      <c r="C128" s="158" t="s">
         <v>18</v>
       </c>
-      <c r="D126" t="s">
-        <v>409</v>
-      </c>
-      <c r="G126" t="s">
+      <c r="G128" s="158" t="s">
         <v>309</v>
       </c>
-      <c r="H126" s="13">
-        <v>45</v>
-      </c>
-      <c r="I126" s="158"/>
-      <c r="J126" s="158"/>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>2</v>
-      </c>
-      <c r="C127" t="s">
-        <v>18</v>
-      </c>
-      <c r="D127" t="s">
-        <v>410</v>
-      </c>
-      <c r="G127" t="s">
-        <v>309</v>
-      </c>
-      <c r="H127" s="13">
-        <v>12</v>
-      </c>
-      <c r="I127" s="158"/>
-      <c r="J127" s="158"/>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>2</v>
-      </c>
-      <c r="C128" t="s">
-        <v>18</v>
-      </c>
-      <c r="D128" t="s">
-        <v>398</v>
-      </c>
-      <c r="G128" t="s">
-        <v>309</v>
-      </c>
-      <c r="H128" s="13">
-        <v>6</v>
+      <c r="H128" s="158">
+        <v>0</v>
       </c>
       <c r="I128" s="158"/>
-      <c r="J128" s="158"/>
+      <c r="J128" s="158" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
@@ -18884,13 +18860,13 @@
         <v>18</v>
       </c>
       <c r="D129" t="s">
-        <v>371</v>
+        <v>409</v>
       </c>
       <c r="G129" t="s">
         <v>309</v>
       </c>
       <c r="H129" s="13">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="I129" s="158"/>
       <c r="J129" s="158"/>
@@ -18903,14 +18879,16 @@
         <v>18</v>
       </c>
       <c r="D130" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="G130" t="s">
         <v>309</v>
       </c>
       <c r="H130" s="13">
-        <v>7</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="I130" s="158"/>
+      <c r="J130" s="158"/>
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
@@ -18920,14 +18898,16 @@
         <v>18</v>
       </c>
       <c r="D131" t="s">
-        <v>466</v>
+        <v>398</v>
       </c>
       <c r="G131" t="s">
         <v>309</v>
       </c>
       <c r="H131" s="13">
-        <v>3</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="I131" s="158"/>
+      <c r="J131" s="158"/>
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
@@ -18937,107 +18917,112 @@
         <v>18</v>
       </c>
       <c r="D132" t="s">
-        <v>403</v>
+        <v>371</v>
       </c>
       <c r="G132" t="s">
         <v>309</v>
       </c>
       <c r="H132" s="13">
+        <v>20</v>
+      </c>
+      <c r="I132" s="158"/>
+      <c r="J132" s="158"/>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>2</v>
+      </c>
+      <c r="C133" t="s">
+        <v>18</v>
+      </c>
+      <c r="D133" t="s">
+        <v>408</v>
+      </c>
+      <c r="G133" t="s">
+        <v>309</v>
+      </c>
+      <c r="H133" s="13">
         <v>7</v>
       </c>
     </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>2</v>
+      </c>
+      <c r="C134" t="s">
+        <v>18</v>
+      </c>
+      <c r="D134" t="s">
+        <v>466</v>
+      </c>
+      <c r="G134" t="s">
+        <v>309</v>
+      </c>
+      <c r="H134" s="13">
+        <v>3</v>
+      </c>
+    </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A135" s="81" t="s">
+      <c r="A135" t="s">
+        <v>2</v>
+      </c>
+      <c r="C135" t="s">
+        <v>18</v>
+      </c>
+      <c r="D135" t="s">
+        <v>403</v>
+      </c>
+      <c r="G135" t="s">
+        <v>309</v>
+      </c>
+      <c r="H135" s="13">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A138" s="81" t="s">
         <v>448</v>
       </c>
-      <c r="B135" s="48"/>
-      <c r="C135" s="49"/>
-      <c r="D135" s="49"/>
-      <c r="E135" s="49"/>
-      <c r="F135" s="49"/>
-      <c r="G135" s="49"/>
-      <c r="H135" s="161"/>
-      <c r="I135" s="49"/>
-      <c r="J135" s="49"/>
-      <c r="K135" s="49"/>
-    </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A136" s="158" t="s">
+      <c r="B138" s="48"/>
+      <c r="C138" s="49"/>
+      <c r="D138" s="49"/>
+      <c r="E138" s="49"/>
+      <c r="F138" s="49"/>
+      <c r="G138" s="49"/>
+      <c r="H138" s="161"/>
+      <c r="I138" s="49"/>
+      <c r="J138" s="49"/>
+      <c r="K138" s="49"/>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A139" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="B136" s="158"/>
-      <c r="C136" s="158"/>
-      <c r="G136" s="158" t="s">
+      <c r="B139" s="158"/>
+      <c r="C139" s="158"/>
+      <c r="G139" s="158" t="s">
         <v>309</v>
       </c>
-      <c r="H136" s="158">
+      <c r="H139" s="158">
         <v>0</v>
       </c>
-      <c r="I136" s="158"/>
-      <c r="J136" s="158" t="s">
+      <c r="I139" s="158"/>
+      <c r="J139" s="158" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>2</v>
-      </c>
-      <c r="D137" t="s">
-        <v>409</v>
-      </c>
-      <c r="G137" t="s">
-        <v>309</v>
-      </c>
-      <c r="H137" s="13">
-        <v>0</v>
-      </c>
-      <c r="I137" s="158"/>
-      <c r="J137" s="158"/>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>2</v>
-      </c>
-      <c r="D138" t="s">
-        <v>410</v>
-      </c>
-      <c r="G138" t="s">
-        <v>309</v>
-      </c>
-      <c r="H138" s="13">
-        <v>55</v>
-      </c>
-      <c r="I138" s="158"/>
-      <c r="J138" s="158"/>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>2</v>
-      </c>
-      <c r="D139" t="s">
-        <v>398</v>
-      </c>
-      <c r="G139" t="s">
-        <v>309</v>
-      </c>
-      <c r="H139" s="13">
-        <v>40</v>
-      </c>
-      <c r="I139" s="158"/>
-      <c r="J139" s="158"/>
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>2</v>
       </c>
       <c r="D140" t="s">
-        <v>371</v>
+        <v>409</v>
       </c>
       <c r="G140" t="s">
         <v>309</v>
       </c>
       <c r="H140" s="13">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I140" s="158"/>
       <c r="J140" s="158"/>
@@ -19047,13 +19032,13 @@
         <v>2</v>
       </c>
       <c r="D141" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="G141" t="s">
         <v>309</v>
       </c>
       <c r="H141" s="13">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="I141" s="158"/>
       <c r="J141" s="158"/>
@@ -19063,13 +19048,13 @@
         <v>2</v>
       </c>
       <c r="D142" t="s">
-        <v>466</v>
+        <v>398</v>
       </c>
       <c r="G142" t="s">
         <v>309</v>
       </c>
       <c r="H142" s="13">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="I142" s="158"/>
       <c r="J142" s="158"/>
@@ -19079,16 +19064,64 @@
         <v>2</v>
       </c>
       <c r="D143" t="s">
-        <v>403</v>
+        <v>371</v>
       </c>
       <c r="G143" t="s">
         <v>309</v>
       </c>
       <c r="H143" s="13">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I143" s="158"/>
       <c r="J143" s="158"/>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>2</v>
+      </c>
+      <c r="D144" t="s">
+        <v>408</v>
+      </c>
+      <c r="G144" t="s">
+        <v>309</v>
+      </c>
+      <c r="H144" s="13">
+        <v>0</v>
+      </c>
+      <c r="I144" s="158"/>
+      <c r="J144" s="158"/>
+    </row>
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>2</v>
+      </c>
+      <c r="D145" t="s">
+        <v>466</v>
+      </c>
+      <c r="G145" t="s">
+        <v>309</v>
+      </c>
+      <c r="H145" s="13">
+        <v>0</v>
+      </c>
+      <c r="I145" s="158"/>
+      <c r="J145" s="158"/>
+    </row>
+    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>2</v>
+      </c>
+      <c r="D146" t="s">
+        <v>403</v>
+      </c>
+      <c r="G146" t="s">
+        <v>309</v>
+      </c>
+      <c r="H146" s="13">
+        <v>0</v>
+      </c>
+      <c r="I146" s="158"/>
+      <c r="J146" s="158"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -25198,49 +25231,49 @@
       </c>
       <c r="AB3" s="198"/>
       <c r="AC3" s="198"/>
-      <c r="AD3" s="268" t="s">
+      <c r="AD3" s="271" t="s">
         <v>508</v>
       </c>
-      <c r="AE3" s="269" t="s">
+      <c r="AE3" s="272" t="s">
         <v>510</v>
       </c>
-      <c r="AF3" s="268" t="s">
+      <c r="AF3" s="271" t="s">
         <v>512</v>
       </c>
-      <c r="AG3" s="269" t="s">
+      <c r="AG3" s="272" t="s">
         <v>514</v>
       </c>
-      <c r="AH3" s="268" t="s">
+      <c r="AH3" s="271" t="s">
         <v>515</v>
       </c>
-      <c r="AI3" s="269" t="s">
+      <c r="AI3" s="272" t="s">
         <v>517</v>
       </c>
-      <c r="AJ3" s="268" t="s">
+      <c r="AJ3" s="271" t="s">
         <v>518</v>
       </c>
-      <c r="AK3" s="269" t="s">
+      <c r="AK3" s="272" t="s">
         <v>519</v>
       </c>
-      <c r="AL3" s="268" t="s">
+      <c r="AL3" s="271" t="s">
         <v>521</v>
       </c>
-      <c r="AM3" s="269" t="s">
+      <c r="AM3" s="272" t="s">
         <v>522</v>
       </c>
-      <c r="AN3" s="268" t="s">
+      <c r="AN3" s="271" t="s">
         <v>542</v>
       </c>
-      <c r="AO3" s="269" t="s">
+      <c r="AO3" s="272" t="s">
         <v>524</v>
       </c>
-      <c r="AP3" s="268" t="s">
+      <c r="AP3" s="271" t="s">
         <v>525</v>
       </c>
-      <c r="AQ3" s="267" t="s">
+      <c r="AQ3" s="270" t="s">
         <v>546</v>
       </c>
-      <c r="AR3" s="266" t="s">
+      <c r="AR3" s="269" t="s">
         <v>541</v>
       </c>
     </row>
@@ -25291,21 +25324,21 @@
       <c r="AA4" s="197"/>
       <c r="AB4" s="198"/>
       <c r="AC4" s="198"/>
-      <c r="AD4" s="268"/>
-      <c r="AE4" s="269"/>
-      <c r="AF4" s="268"/>
-      <c r="AG4" s="269"/>
-      <c r="AH4" s="268"/>
-      <c r="AI4" s="269"/>
-      <c r="AJ4" s="268"/>
-      <c r="AK4" s="269"/>
-      <c r="AL4" s="268"/>
-      <c r="AM4" s="269"/>
-      <c r="AN4" s="268"/>
-      <c r="AO4" s="269"/>
-      <c r="AP4" s="268"/>
-      <c r="AQ4" s="267"/>
-      <c r="AR4" s="266"/>
+      <c r="AD4" s="271"/>
+      <c r="AE4" s="272"/>
+      <c r="AF4" s="271"/>
+      <c r="AG4" s="272"/>
+      <c r="AH4" s="271"/>
+      <c r="AI4" s="272"/>
+      <c r="AJ4" s="271"/>
+      <c r="AK4" s="272"/>
+      <c r="AL4" s="271"/>
+      <c r="AM4" s="272"/>
+      <c r="AN4" s="271"/>
+      <c r="AO4" s="272"/>
+      <c r="AP4" s="271"/>
+      <c r="AQ4" s="270"/>
+      <c r="AR4" s="269"/>
     </row>
     <row r="5" spans="2:44" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="205" t="s">
@@ -25386,21 +25419,21 @@
       <c r="AA5" s="197"/>
       <c r="AB5" s="198"/>
       <c r="AC5" s="198"/>
-      <c r="AD5" s="268"/>
-      <c r="AE5" s="269"/>
-      <c r="AF5" s="268"/>
-      <c r="AG5" s="269"/>
-      <c r="AH5" s="268"/>
-      <c r="AI5" s="269"/>
-      <c r="AJ5" s="268"/>
-      <c r="AK5" s="269"/>
-      <c r="AL5" s="268"/>
-      <c r="AM5" s="269"/>
-      <c r="AN5" s="268"/>
-      <c r="AO5" s="269"/>
-      <c r="AP5" s="268"/>
-      <c r="AQ5" s="267"/>
-      <c r="AR5" s="266" t="s">
+      <c r="AD5" s="271"/>
+      <c r="AE5" s="272"/>
+      <c r="AF5" s="271"/>
+      <c r="AG5" s="272"/>
+      <c r="AH5" s="271"/>
+      <c r="AI5" s="272"/>
+      <c r="AJ5" s="271"/>
+      <c r="AK5" s="272"/>
+      <c r="AL5" s="271"/>
+      <c r="AM5" s="272"/>
+      <c r="AN5" s="271"/>
+      <c r="AO5" s="272"/>
+      <c r="AP5" s="271"/>
+      <c r="AQ5" s="270"/>
+      <c r="AR5" s="269" t="s">
         <v>540</v>
       </c>
     </row>
@@ -26835,23 +26868,23 @@
       <c r="N23" s="167"/>
       <c r="O23" s="167"/>
       <c r="P23" s="167"/>
-      <c r="Q23" s="271" t="s">
+      <c r="Q23" s="268" t="s">
         <v>560</v>
       </c>
-      <c r="R23" s="271" t="s">
+      <c r="R23" s="268" t="s">
         <v>561</v>
       </c>
-      <c r="S23" s="271" t="s">
+      <c r="S23" s="268" t="s">
         <v>548</v>
       </c>
-      <c r="T23" s="270" t="s">
+      <c r="T23" s="267" t="s">
         <v>290</v>
       </c>
-      <c r="U23" s="270"/>
-      <c r="V23" s="270" t="s">
+      <c r="U23" s="267"/>
+      <c r="V23" s="267" t="s">
         <v>291</v>
       </c>
-      <c r="W23" s="270"/>
+      <c r="W23" s="267"/>
       <c r="X23" s="166" t="s">
         <v>453</v>
       </c>
@@ -26876,9 +26909,9 @@
       <c r="P24" s="168" t="s">
         <v>454</v>
       </c>
-      <c r="Q24" s="271"/>
-      <c r="R24" s="271"/>
-      <c r="S24" s="271"/>
+      <c r="Q24" s="268"/>
+      <c r="R24" s="268"/>
+      <c r="S24" s="268"/>
       <c r="T24" s="240" t="s">
         <v>454</v>
       </c>
@@ -33675,11 +33708,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="V23:W23"/>
-    <mergeCell ref="T23:U23"/>
-    <mergeCell ref="Q23:Q24"/>
-    <mergeCell ref="R23:R24"/>
-    <mergeCell ref="S23:S24"/>
     <mergeCell ref="AR3:AR5"/>
     <mergeCell ref="AQ3:AQ5"/>
     <mergeCell ref="AD3:AD5"/>
@@ -33695,6 +33723,11 @@
     <mergeCell ref="AN3:AN5"/>
     <mergeCell ref="AO3:AO5"/>
     <mergeCell ref="AP3:AP5"/>
+    <mergeCell ref="V23:W23"/>
+    <mergeCell ref="T23:U23"/>
+    <mergeCell ref="Q23:Q24"/>
+    <mergeCell ref="R23:R24"/>
+    <mergeCell ref="S23:S24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>